<commit_message>
feat(mapping)!: replace existing external mappings instead of adding to them (DEV-6897) (#2386)
Co-authored-by: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/testdata/mapping/4124_testonto_Mapping_good.xlsx
+++ b/testdata/mapping/4124_testonto_Mapping_good.xlsx
@@ -1,126 +1,50 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11028"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/noraammann/Downloads/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C75016BB-130F-FA46-AE55-7BA161D5AC25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6320" yWindow="2980" windowWidth="28240" windowHeight="17240" activeTab="2" xr2:uid="{0F3E081E-C864-8640-9A73-45072465AE86}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="6320" yWindow="2980" windowWidth="28240" windowHeight="17240" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="prefix" sheetId="1" r:id="rId1"/>
-    <sheet name="classes" sheetId="2" r:id="rId2"/>
-    <sheet name="properties" sheetId="6" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="prefix" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="classes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="properties" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="181029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="181029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="17">
-  <si>
-    <t>property</t>
-  </si>
-  <si>
-    <t>mapping</t>
-  </si>
-  <si>
-    <t>prefix</t>
-  </si>
-  <si>
-    <t>dcterms</t>
-  </si>
-  <si>
-    <t>class</t>
-  </si>
-  <si>
-    <t>https://www.dublincore.org/specifications/dublin-core/dcmi-terms/</t>
-  </si>
-  <si>
-    <t>schema</t>
-  </si>
-  <si>
-    <t>https://www.w3.org/TR/rdf-schema/</t>
-  </si>
-  <si>
-    <t>cidoc</t>
-  </si>
-  <si>
-    <t>bibo</t>
-  </si>
-  <si>
-    <t>http://purl.org/ontology/bibo/</t>
-  </si>
-  <si>
-    <t>http://www.cidoc-crm.org/cidoc-crm/</t>
-  </si>
-  <si>
-    <t>cidoc:E22_Human-Made_Object; schema:Book; bibo:Book</t>
-  </si>
-  <si>
-    <t>dcterms:title</t>
-  </si>
-  <si>
-    <t>link</t>
-  </si>
-  <si>
-    <t>minimalResource</t>
-  </si>
-  <si>
-    <t>hasText</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="3">
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="12"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <name val="Aptos Narrow"/>
+      <b val="1"/>
+      <color theme="1"/>
       <sz val="12"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="12"/>
-      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <color theme="10"/>
+      <sz val="12"/>
+      <u val="single"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -137,27 +61,86 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -477,123 +460,195 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EDBE472B-D79E-E843-9C88-7AC0BC1D8BD5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B5"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
-    <col min="1" max="1" width="12.6640625" customWidth="1"/>
-    <col min="2" max="2" width="58.33203125" customWidth="1"/>
+    <col width="12.6640625" customWidth="1" min="1" max="1"/>
+    <col width="58.33203125" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>10</v>
+    <row r="1" customFormat="1" s="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>prefix</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>dcterms</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dublincore.org/specifications/dublin-core/dcmi-terms/</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>schema</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.w3.org/TR/rdf-schema/</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>cidoc</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>http://www.cidoc-crm.org/cidoc-crm/</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>bibo</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>http://purl.org/ontology/bibo/</t>
+        </is>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1" xr:uid="{5AB1213F-2E75-8B42-A1ED-C483D742895E}"/>
-    <hyperlink ref="B3" r:id="rId2" xr:uid="{5515930E-9C2C-E94E-BFCA-D14166AAE81D}"/>
-    <hyperlink ref="B5" r:id="rId3" xr:uid="{C558E2EC-E5F8-9247-BD96-E2B15F50E932}"/>
-    <hyperlink ref="B4" r:id="rId4" xr:uid="{076F7D93-A7A7-BA40-ABEE-66F50C777997}"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId4"/>
   </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageMargins left="0.7" right="0.7" top="0.787401575" bottom="0.787401575" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D106943-1610-8549-B7DF-5339A1B61DDA}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
-    <col min="1" max="1" width="15.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="54" customWidth="1"/>
+    <col width="15.33203125" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="54" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B2" t="s">
-        <v>12</v>
+    <row r="1" customFormat="1" s="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>class</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>mapping</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>minimalResource</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>cidoc:E22_Human-Made_Object; schema:Book; bibo:Book</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>otherResource</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>cidoc:E21_Person</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+  <pageMargins left="0.7" right="0.7" top="0.787401575" bottom="0.787401575" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{143185D6-C43E-E946-9AA9-F24EEF8275AE}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
-    <col min="1" max="1" width="22.83203125" customWidth="1"/>
-    <col min="2" max="2" width="75" customWidth="1"/>
+    <col width="22.83203125" customWidth="1" min="1" max="1"/>
+    <col width="75" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B2" t="s">
-        <v>13</v>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>property</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>mapping</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>hasText</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>dcterms:title</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>hasOtherText</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>dcterms:description</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+  <pageMargins left="0.7" right="0.7" top="0.787401575" bottom="0.787401575" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>